<commit_message>
Updated ITA_grids_kan model - 2025-12-05 21:44
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_ITA_grids_kan/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{61222A17-D04D-428E-929F-6EDD4703898E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A31FB39-DF9E-4721-88D5-808EE634389E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3113,7 +3113,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DC264C9-7237-4E4F-BE31-EC6A1F55BC86}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EBACB81-A929-4F5B-941C-CE85FF2F2ADD}">
   <dimension ref="B9:E331"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids_kan model - 2025-12-08 12:33
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_ITA_grids_kan/Sets-vervestacks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A31FB39-DF9E-4721-88D5-808EE634389E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B43CD18B-AA1D-4090-8AC5-AB65F49DBCBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2940" yWindow="2940" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -3113,7 +3113,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EBACB81-A929-4F5B-941C-CE85FF2F2ADD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84196ED7-AE68-475E-A894-74526BC92582}">
   <dimension ref="B9:E331"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated ITA_grids_kan model - 2025-12-11 12:20
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_ITA_grids_kan/Sets-vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B43CD18B-AA1D-4090-8AC5-AB65F49DBCBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D3FB65C6-25CB-4274-9919-232B806AAF57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2940" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -3113,7 +3113,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84196ED7-AE68-475E-A894-74526BC92582}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{077DB8B4-AD7F-4C92-AB49-68A7996CF39A}">
   <dimension ref="B9:E331"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>